<commit_message>
rilevazioen A OK? + campioni B OK TODO check A, qualitative B, spese B
</commit_message>
<xml_diff>
--- a/analisi_spese_sottocampioni.xlsx
+++ b/analisi_spese_sottocampioni.xlsx
@@ -10959,7 +10959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11054,25 +11054,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>487.2683</v>
+        <v>536</v>
       </c>
       <c r="D6" t="n">
-        <v>32.439</v>
+        <v>31.6667</v>
       </c>
       <c r="E6" t="n">
-        <v>193.9024</v>
+        <v>208.3333</v>
       </c>
       <c r="F6" t="n">
-        <v>57.8049</v>
+        <v>95</v>
       </c>
       <c r="G6" t="n">
-        <v>162.9268</v>
+        <v>158.3333</v>
       </c>
       <c r="H6" t="n">
-        <v>10.2439</v>
+        <v>1.6667</v>
       </c>
       <c r="I6" t="n">
-        <v>29.9512</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7">
@@ -11087,25 +11087,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>730.6818</v>
+        <v>992</v>
       </c>
       <c r="D7" t="n">
-        <v>46.7045</v>
+        <v>20</v>
       </c>
       <c r="E7" t="n">
-        <v>266.8182</v>
+        <v>425</v>
       </c>
       <c r="F7" t="n">
-        <v>60.2273</v>
+        <v>142</v>
       </c>
       <c r="G7" t="n">
-        <v>287.5</v>
+        <v>290</v>
       </c>
       <c r="H7" t="n">
-        <v>10.5682</v>
+        <v>15</v>
       </c>
       <c r="I7" t="n">
-        <v>58.8636</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -11120,25 +11120,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>613.2705999999999</v>
+        <v>743.2727</v>
       </c>
       <c r="D8" t="n">
-        <v>39.8235</v>
+        <v>26.3636</v>
       </c>
       <c r="E8" t="n">
-        <v>231.6471</v>
+        <v>306.8182</v>
       </c>
       <c r="F8" t="n">
-        <v>59.0588</v>
+        <v>116.3636</v>
       </c>
       <c r="G8" t="n">
-        <v>227.4118</v>
+        <v>218.1818</v>
       </c>
       <c r="H8" t="n">
-        <v>10.4118</v>
+        <v>7.7273</v>
       </c>
       <c r="I8" t="n">
-        <v>44.9176</v>
+        <v>67.8182</v>
       </c>
     </row>
     <row r="10">
@@ -11207,25 +11207,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>88.7911</v>
+        <v>89.33329999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>5.9111</v>
+        <v>5.2778</v>
       </c>
       <c r="E12" t="n">
-        <v>35.3333</v>
+        <v>34.7222</v>
       </c>
       <c r="F12" t="n">
-        <v>10.5333</v>
+        <v>15.8333</v>
       </c>
       <c r="G12" t="n">
-        <v>29.6889</v>
+        <v>26.3889</v>
       </c>
       <c r="H12" t="n">
-        <v>1.8667</v>
+        <v>0.2778</v>
       </c>
       <c r="I12" t="n">
-        <v>5.4578</v>
+        <v>6.8333</v>
       </c>
     </row>
     <row r="13">
@@ -11240,25 +11240,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>100.4688</v>
+        <v>101.2245</v>
       </c>
       <c r="D13" t="n">
-        <v>6.4219</v>
+        <v>2.0408</v>
       </c>
       <c r="E13" t="n">
-        <v>36.6875</v>
+        <v>43.3673</v>
       </c>
       <c r="F13" t="n">
-        <v>8.2812</v>
+        <v>14.4898</v>
       </c>
       <c r="G13" t="n">
-        <v>39.5312</v>
+        <v>29.5918</v>
       </c>
       <c r="H13" t="n">
-        <v>1.4531</v>
+        <v>1.5306</v>
       </c>
       <c r="I13" t="n">
-        <v>8.0938</v>
+        <v>10.2041</v>
       </c>
     </row>
     <row r="14">
@@ -11273,25 +11273,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>95.6477</v>
+        <v>96.18819999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>6.211</v>
+        <v>3.4118</v>
       </c>
       <c r="E14" t="n">
-        <v>36.1284</v>
+        <v>39.7059</v>
       </c>
       <c r="F14" t="n">
-        <v>9.211</v>
+        <v>15.0588</v>
       </c>
       <c r="G14" t="n">
-        <v>35.4679</v>
+        <v>28.2353</v>
       </c>
       <c r="H14" t="n">
-        <v>1.6239</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>7.0055</v>
+        <v>8.7765</v>
       </c>
     </row>
     <row r="16">
@@ -11360,25 +11360,25 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>811.3882</v>
+        <v>582</v>
       </c>
       <c r="D18" t="n">
-        <v>65.5882</v>
+        <v>20.5</v>
       </c>
       <c r="E18" t="n">
-        <v>456.6471</v>
+        <v>296</v>
       </c>
       <c r="F18" t="n">
-        <v>122.5882</v>
+        <v>58</v>
       </c>
       <c r="G18" t="n">
-        <v>138</v>
+        <v>177</v>
       </c>
       <c r="H18" t="n">
-        <v>14.6471</v>
+        <v>19</v>
       </c>
       <c r="I18" t="n">
-        <v>13.9176</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="19">
@@ -11393,22 +11393,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1416.3</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>182.8</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>128.5</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>315</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -11426,25 +11426,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>811.3882</v>
+        <v>999.15</v>
       </c>
       <c r="D20" t="n">
-        <v>65.5882</v>
+        <v>101.65</v>
       </c>
       <c r="E20" t="n">
-        <v>456.6471</v>
+        <v>523</v>
       </c>
       <c r="F20" t="n">
-        <v>122.5882</v>
+        <v>93.25</v>
       </c>
       <c r="G20" t="n">
-        <v>138</v>
+        <v>246</v>
       </c>
       <c r="H20" t="n">
-        <v>14.6471</v>
+        <v>29.5</v>
       </c>
       <c r="I20" t="n">
-        <v>13.9176</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="22">
@@ -11513,25 +11513,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>56.7638</v>
+        <v>71.8519</v>
       </c>
       <c r="D24" t="n">
-        <v>4.5885</v>
+        <v>2.5309</v>
       </c>
       <c r="E24" t="n">
-        <v>31.9465</v>
+        <v>36.5432</v>
       </c>
       <c r="F24" t="n">
-        <v>8.5761</v>
+        <v>7.1605</v>
       </c>
       <c r="G24" t="n">
-        <v>9.654299999999999</v>
+        <v>21.8519</v>
       </c>
       <c r="H24" t="n">
-        <v>1.0247</v>
+        <v>2.3457</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9737</v>
+        <v>1.4198</v>
       </c>
     </row>
     <row r="25">
@@ -11546,22 +11546,22 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>214.5909</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>27.697</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>113.6364</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>19.4697</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>47.7273</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>6.0606</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -11579,25 +11579,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>56.7638</v>
+        <v>135.9388</v>
       </c>
       <c r="D26" t="n">
-        <v>4.5885</v>
+        <v>13.8299</v>
       </c>
       <c r="E26" t="n">
-        <v>31.9465</v>
+        <v>71.15649999999999</v>
       </c>
       <c r="F26" t="n">
-        <v>8.5761</v>
+        <v>12.6871</v>
       </c>
       <c r="G26" t="n">
-        <v>9.654299999999999</v>
+        <v>33.4694</v>
       </c>
       <c r="H26" t="n">
-        <v>1.0247</v>
+        <v>4.0136</v>
       </c>
       <c r="I26" t="n">
-        <v>0.9737</v>
+        <v>0.7823</v>
       </c>
     </row>
     <row r="28">
@@ -11666,25 +11666,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>386.6216</v>
+        <v>460.3</v>
       </c>
       <c r="D30" t="n">
-        <v>47.1351</v>
+        <v>119</v>
       </c>
       <c r="E30" t="n">
-        <v>122.973</v>
+        <v>127</v>
       </c>
       <c r="F30" t="n">
-        <v>33.4324</v>
+        <v>51</v>
       </c>
       <c r="G30" t="n">
-        <v>143.9189</v>
+        <v>127</v>
       </c>
       <c r="H30" t="n">
-        <v>17.9189</v>
+        <v>10.3</v>
       </c>
       <c r="I30" t="n">
-        <v>21.2432</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31">
@@ -11699,25 +11699,25 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>829.4468000000001</v>
+        <v>699.7</v>
       </c>
       <c r="D31" t="n">
-        <v>64.89360000000001</v>
+        <v>70</v>
       </c>
       <c r="E31" t="n">
-        <v>354.9362</v>
+        <v>252.2</v>
       </c>
       <c r="F31" t="n">
-        <v>100.7021</v>
+        <v>113.5</v>
       </c>
       <c r="G31" t="n">
-        <v>277.4468</v>
+        <v>248</v>
       </c>
       <c r="H31" t="n">
-        <v>18.0851</v>
+        <v>11</v>
       </c>
       <c r="I31" t="n">
-        <v>13.383</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32">
@@ -11732,25 +11732,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>634.3929000000001</v>
+        <v>580</v>
       </c>
       <c r="D32" t="n">
-        <v>57.0714</v>
+        <v>94.5</v>
       </c>
       <c r="E32" t="n">
-        <v>252.7619</v>
+        <v>189.6</v>
       </c>
       <c r="F32" t="n">
-        <v>71.0714</v>
+        <v>82.25</v>
       </c>
       <c r="G32" t="n">
-        <v>218.631</v>
+        <v>187.5</v>
       </c>
       <c r="H32" t="n">
-        <v>18.0119</v>
+        <v>10.65</v>
       </c>
       <c r="I32" t="n">
-        <v>16.8452</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="34">
@@ -11819,25 +11819,25 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>75.2895</v>
+        <v>74.2419</v>
       </c>
       <c r="D36" t="n">
-        <v>9.178900000000001</v>
+        <v>19.1935</v>
       </c>
       <c r="E36" t="n">
-        <v>23.9474</v>
+        <v>20.4839</v>
       </c>
       <c r="F36" t="n">
-        <v>6.5105</v>
+        <v>8.2258</v>
       </c>
       <c r="G36" t="n">
-        <v>28.0263</v>
+        <v>20.4839</v>
       </c>
       <c r="H36" t="n">
-        <v>3.4895</v>
+        <v>1.6613</v>
       </c>
       <c r="I36" t="n">
-        <v>4.1368</v>
+        <v>4.1935</v>
       </c>
     </row>
     <row r="37">
@@ -11852,25 +11852,25 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>85.67910000000001</v>
+        <v>134.5577</v>
       </c>
       <c r="D37" t="n">
-        <v>6.7033</v>
+        <v>13.4615</v>
       </c>
       <c r="E37" t="n">
-        <v>36.6637</v>
+        <v>48.5</v>
       </c>
       <c r="F37" t="n">
-        <v>10.4022</v>
+        <v>21.8269</v>
       </c>
       <c r="G37" t="n">
-        <v>28.6593</v>
+        <v>47.6923</v>
       </c>
       <c r="H37" t="n">
-        <v>1.8681</v>
+        <v>2.1154</v>
       </c>
       <c r="I37" t="n">
-        <v>1.3824</v>
+        <v>0.9615</v>
       </c>
     </row>
     <row r="38">
@@ -11885,25 +11885,25 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>82.6186</v>
+        <v>101.7544</v>
       </c>
       <c r="D38" t="n">
-        <v>7.4326</v>
+        <v>16.5789</v>
       </c>
       <c r="E38" t="n">
-        <v>32.9178</v>
+        <v>33.2632</v>
       </c>
       <c r="F38" t="n">
-        <v>9.255800000000001</v>
+        <v>14.4298</v>
       </c>
       <c r="G38" t="n">
-        <v>28.4729</v>
+        <v>32.8947</v>
       </c>
       <c r="H38" t="n">
-        <v>2.3457</v>
+        <v>1.8684</v>
       </c>
       <c r="I38" t="n">
-        <v>2.1938</v>
+        <v>2.7193</v>
       </c>
     </row>
     <row r="40">
@@ -11972,25 +11972,25 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>414.678</v>
+        <v>503.2727</v>
       </c>
       <c r="D42" t="n">
-        <v>27.4915</v>
+        <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>155.0508</v>
+        <v>150</v>
       </c>
       <c r="F42" t="n">
-        <v>32.3729</v>
+        <v>30</v>
       </c>
       <c r="G42" t="n">
-        <v>165.0847</v>
+        <v>270</v>
       </c>
       <c r="H42" t="n">
-        <v>4.322</v>
+        <v>8.181800000000001</v>
       </c>
       <c r="I42" t="n">
-        <v>30.3559</v>
+        <v>45.0909</v>
       </c>
     </row>
     <row r="43">
@@ -12005,25 +12005,25 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>853.6538</v>
+        <v>1367.5</v>
       </c>
       <c r="D43" t="n">
-        <v>107.3077</v>
+        <v>159</v>
       </c>
       <c r="E43" t="n">
-        <v>341.9231</v>
+        <v>538</v>
       </c>
       <c r="F43" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="G43" t="n">
-        <v>248.0769</v>
+        <v>380</v>
       </c>
       <c r="H43" t="n">
-        <v>23.8462</v>
+        <v>50</v>
       </c>
       <c r="I43" t="n">
-        <v>77.5</v>
+        <v>167.5</v>
       </c>
     </row>
     <row r="44">
@@ -12038,25 +12038,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>548.9529</v>
+        <v>914.8095</v>
       </c>
       <c r="D44" t="n">
-        <v>51.9059</v>
+        <v>75.71429999999999</v>
       </c>
       <c r="E44" t="n">
-        <v>212.2118</v>
+        <v>334.7619</v>
       </c>
       <c r="F44" t="n">
-        <v>39.2941</v>
+        <v>50.4762</v>
       </c>
       <c r="G44" t="n">
-        <v>190.4706</v>
+        <v>322.381</v>
       </c>
       <c r="H44" t="n">
-        <v>10.2941</v>
+        <v>28.0952</v>
       </c>
       <c r="I44" t="n">
-        <v>44.7765</v>
+        <v>103.381</v>
       </c>
     </row>
     <row r="46">
@@ -12125,25 +12125,25 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>47.05</v>
+        <v>51.7383</v>
       </c>
       <c r="D48" t="n">
-        <v>3.1192</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>17.5923</v>
+        <v>15.4206</v>
       </c>
       <c r="F48" t="n">
-        <v>3.6731</v>
+        <v>3.0841</v>
       </c>
       <c r="G48" t="n">
-        <v>18.7308</v>
+        <v>27.757</v>
       </c>
       <c r="H48" t="n">
-        <v>0.4904</v>
+        <v>0.8411</v>
       </c>
       <c r="I48" t="n">
-        <v>3.4442</v>
+        <v>4.6355</v>
       </c>
     </row>
     <row r="49">
@@ -12158,25 +12158,25 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>111.5327</v>
+        <v>155.3977</v>
       </c>
       <c r="D49" t="n">
-        <v>14.0201</v>
+        <v>18.0682</v>
       </c>
       <c r="E49" t="n">
-        <v>44.6734</v>
+        <v>61.1364</v>
       </c>
       <c r="F49" t="n">
-        <v>7.1859</v>
+        <v>8.295500000000001</v>
       </c>
       <c r="G49" t="n">
-        <v>32.4121</v>
+        <v>43.1818</v>
       </c>
       <c r="H49" t="n">
-        <v>3.1156</v>
+        <v>5.6818</v>
       </c>
       <c r="I49" t="n">
-        <v>10.1256</v>
+        <v>19.0341</v>
       </c>
     </row>
     <row r="50">
@@ -12191,25 +12191,25 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>64.89709999999999</v>
+        <v>98.5179</v>
       </c>
       <c r="D50" t="n">
-        <v>6.1363</v>
+        <v>8.1538</v>
       </c>
       <c r="E50" t="n">
-        <v>25.0876</v>
+        <v>36.0513</v>
       </c>
       <c r="F50" t="n">
-        <v>4.6453</v>
+        <v>5.4359</v>
       </c>
       <c r="G50" t="n">
-        <v>22.5174</v>
+        <v>34.7179</v>
       </c>
       <c r="H50" t="n">
-        <v>1.217</v>
+        <v>3.0256</v>
       </c>
       <c r="I50" t="n">
-        <v>5.2935</v>
+        <v>11.1333</v>
       </c>
     </row>
     <row r="52">
@@ -12278,25 +12278,25 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>333.4118</v>
+        <v>316.7</v>
       </c>
       <c r="D54" t="n">
-        <v>13.6824</v>
+        <v>39</v>
       </c>
       <c r="E54" t="n">
-        <v>71.05880000000001</v>
+        <v>80</v>
       </c>
       <c r="F54" t="n">
-        <v>78.96469999999999</v>
+        <v>53.7</v>
       </c>
       <c r="G54" t="n">
-        <v>140.4118</v>
+        <v>106.5</v>
       </c>
       <c r="H54" t="n">
-        <v>18.0118</v>
+        <v>35</v>
       </c>
       <c r="I54" t="n">
-        <v>11.2824</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="55">
@@ -12311,25 +12311,25 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>544</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="E55" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56">
@@ -12344,25 +12344,25 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>333.4118</v>
+        <v>430.35</v>
       </c>
       <c r="D56" t="n">
-        <v>13.6824</v>
+        <v>79</v>
       </c>
       <c r="E56" t="n">
-        <v>71.05880000000001</v>
+        <v>72.5</v>
       </c>
       <c r="F56" t="n">
-        <v>78.96469999999999</v>
+        <v>96.34999999999999</v>
       </c>
       <c r="G56" t="n">
-        <v>140.4118</v>
+        <v>133.25</v>
       </c>
       <c r="H56" t="n">
-        <v>18.0118</v>
+        <v>25.5</v>
       </c>
       <c r="I56" t="n">
-        <v>11.2824</v>
+        <v>23.75</v>
       </c>
     </row>
     <row r="58">
@@ -12431,25 +12431,25 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>31.3149</v>
+        <v>49.4844</v>
       </c>
       <c r="D60" t="n">
-        <v>1.2851</v>
+        <v>6.0938</v>
       </c>
       <c r="E60" t="n">
-        <v>6.674</v>
+        <v>12.5</v>
       </c>
       <c r="F60" t="n">
-        <v>7.4166</v>
+        <v>8.390599999999999</v>
       </c>
       <c r="G60" t="n">
-        <v>13.1878</v>
+        <v>16.6406</v>
       </c>
       <c r="H60" t="n">
-        <v>1.6917</v>
+        <v>5.4688</v>
       </c>
       <c r="I60" t="n">
-        <v>1.0597</v>
+        <v>0.3906</v>
       </c>
     </row>
     <row r="61">
@@ -12464,25 +12464,25 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>55.5102</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>12.1429</v>
       </c>
       <c r="E61" t="n">
-        <v>0</v>
+        <v>6.6327</v>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
+        <v>14.1837</v>
       </c>
       <c r="G61" t="n">
-        <v>0</v>
+        <v>16.3265</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>1.6327</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>4.5918</v>
       </c>
     </row>
     <row r="62">
@@ -12497,25 +12497,1050 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>31.3149</v>
+        <v>53.1296</v>
       </c>
       <c r="D62" t="n">
-        <v>1.2851</v>
+        <v>9.7531</v>
       </c>
       <c r="E62" t="n">
-        <v>6.674</v>
+        <v>8.9506</v>
       </c>
       <c r="F62" t="n">
-        <v>7.4166</v>
+        <v>11.8951</v>
       </c>
       <c r="G62" t="n">
-        <v>13.1878</v>
+        <v>16.4506</v>
       </c>
       <c r="H62" t="n">
-        <v>1.6917</v>
+        <v>3.1481</v>
       </c>
       <c r="I62" t="n">
-        <v>1.0597</v>
+        <v>2.9321</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>2. Relazione tra gradi di giudizio, motivazione principale e STP/STPG totale</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Tabella STP</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>motivazione_principale</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>giudizio</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>gruppo</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>totale</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>509.2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>509.2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>938.3333</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1462.5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>811.25</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>687.5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1404.75</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1046.125</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>757.8333</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>757.8333</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>460.3</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>612.5</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>503.7857</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>RURALE E NATURALISTICO</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>503.2727</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>RURALE E NATURALISTICO</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>1367.5</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>RURALE E NATURALISTICO</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>914.8095</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>505.5</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>505.5</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>190.8333</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>411.5625</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Tabella STPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>motivazione_principale</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>giudizio</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>gruppo</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>totale</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>87.7931</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>87.7931</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>95.71429999999999</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>101.2245</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ATTIVO O SPORTIVO</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>100.5357</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>22.8571</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>146.25</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>95.44119999999999</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>82.0896</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>244.3043</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>BALNEARE</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>148.1239</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>206.6818</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>206.6818</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>74.2419</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>81.66670000000001</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>CULTURALE - MUSEALE (ARTISTICO E ARCHITETTONICO)</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>76.663</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>RURALE E NATURALISTICO</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>51.7383</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>RURALE E NATURALISTICO</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>155.3977</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>RURALE E NATURALISTICO</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>98.5179</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>67.40000000000001</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>BUONO</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>67.40000000000001</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>ITALIANI</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>33.6765</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>STRANIERI</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>55.5102</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>VISITA A PARENTI E/O AMICI</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>OTTIMO</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>49.8864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>